<commit_message>
add video trace overlay and peak detection
</commit_message>
<xml_diff>
--- a/PFC/EPM_Center_point/Preinduction/Export Files/Statistics-EPM_preinduction_BigArena_his_res.xlsx
+++ b/PFC/EPM_Center_point/Preinduction/Export Files/Statistics-EPM_preinduction_BigArena_his_res.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annastuckert/Downloads/Git_repositories/FP_behaviour_analysis/PFC/EPM_Center_point/Preinduction/Export Files/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_56168B5F8DF6AE8BD5781DDE33BFE4E7CC94EF40" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="90" windowWidth="17115" windowHeight="9465"/>
+    <workbookView xWindow="10080" yWindow="600" windowWidth="17120" windowHeight="9460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis" sheetId="1" r:id="rId1"/>
@@ -14,55 +20,302 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>column 1</t>
-  </si>
-  <si>
-    <t>column 2</t>
-  </si>
-  <si>
-    <t>column 3</t>
-  </si>
-  <si>
-    <t>column 4</t>
-  </si>
-  <si>
-    <t>column 5</t>
-  </si>
-  <si>
-    <t>column 6</t>
-  </si>
-  <si>
-    <t>column 7</t>
-  </si>
-  <si>
-    <t>column 8</t>
-  </si>
-  <si>
-    <t>column 9</t>
-  </si>
-  <si>
-    <t>column10</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="96">
+  <si>
+    <t>Trial</t>
+  </si>
+  <si>
+    <t>Cagenumber and earmark</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>FP file</t>
+  </si>
+  <si>
+    <t>Cohort</t>
+  </si>
+  <si>
+    <t>Distance moved Center-point Total cm</t>
+  </si>
+  <si>
+    <t>Velocity Center-point Mean cm/s</t>
+  </si>
+  <si>
+    <t>In zone 2 Arena / Center-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 2 Arena / Center-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 2 Arena / Center-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 2 O1_prevC1 / Center-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 2 O1_prevC1 / Center-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 2 O1_prevC1 / Center-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 2 O2_prevC2 / Center-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 2 O2_prevC2 / Center-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 2 O2_prevC2 / Center-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 2 C1_prevO1 / Center-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 2 C1_prevO1 / Center-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 2 C1_prevO1 / Center-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 2 C2_prevO2 / Center-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 2 C2_prevO2 / Center-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 2 C2_prevO2 / Center-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 2 NeutralZone / Center-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 2 NeutralZone / Center-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 2 NeutralZone / Center-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 Arena / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 Arena / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 Arena / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 O1_prevC1 / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 O1_prevC1 / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 O1_prevC1 / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 O2_prevC2 / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 O2_prevC2 / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 O2_prevC2 / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 C1_prevO1 / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 C1_prevO1 / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 C1_prevO1 / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 C2_prevO2 / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 C2_prevO2 / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 C2_prevO2 / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 NeutralZone / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 NeutralZone / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 NeutralZone / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 O1_round / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 O1_round / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 O1_round / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>In zone 3 O2_round / Nose-point Frequency</t>
+  </si>
+  <si>
+    <t>In zone 3 O2_round / Nose-point Cumulative Duration s</t>
+  </si>
+  <si>
+    <t>In zone 3 O2_round / Nose-point Latency to First s</t>
+  </si>
+  <si>
+    <t>Trial     1</t>
+  </si>
+  <si>
+    <t>9E10</t>
+  </si>
+  <si>
+    <t>376</t>
+  </si>
+  <si>
+    <t>EPM_FP0_1</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Trial     2</t>
+  </si>
+  <si>
+    <t>9E3</t>
+  </si>
+  <si>
+    <t>372</t>
+  </si>
+  <si>
+    <t>EPM_FP1_1</t>
+  </si>
+  <si>
+    <t>Trial     3</t>
+  </si>
+  <si>
+    <t>8E4</t>
+  </si>
+  <si>
+    <t>374</t>
+  </si>
+  <si>
+    <t>EPM_FP2_1</t>
+  </si>
+  <si>
+    <t>Trial     4</t>
+  </si>
+  <si>
+    <t>10E13</t>
+  </si>
+  <si>
+    <t>429</t>
+  </si>
+  <si>
+    <t>EPM_FP3_1</t>
+  </si>
+  <si>
+    <t>Trial     5</t>
+  </si>
+  <si>
+    <t>10E4</t>
+  </si>
+  <si>
+    <t>423</t>
+  </si>
+  <si>
+    <t>EPM_FP5_1</t>
+  </si>
+  <si>
+    <t>Trial     6</t>
+  </si>
+  <si>
+    <t>8C4</t>
+  </si>
+  <si>
+    <t>461</t>
+  </si>
+  <si>
+    <t>EPM_FP_00_2</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Trial     7</t>
+  </si>
+  <si>
+    <t>8C10</t>
+  </si>
+  <si>
+    <t>463</t>
+  </si>
+  <si>
+    <t>EPM_FP_0_2</t>
+  </si>
+  <si>
+    <t>Trial     8</t>
+  </si>
+  <si>
+    <t>8C3</t>
+  </si>
+  <si>
+    <t>459</t>
+  </si>
+  <si>
+    <t>EPM_FP_1_2</t>
+  </si>
+  <si>
+    <t>Trial     9</t>
+  </si>
+  <si>
+    <t>5B1</t>
+  </si>
+  <si>
+    <t>398</t>
+  </si>
+  <si>
+    <t>EPM_FP_3_2</t>
+  </si>
+  <si>
+    <t>Trial    10</t>
+  </si>
+  <si>
+    <t>5B3</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>EPM_FP_4_2</t>
+  </si>
+  <si>
+    <t>Trial    11</t>
+  </si>
+  <si>
+    <t>5B4</t>
+  </si>
+  <si>
+    <t>402</t>
+  </si>
+  <si>
+    <t>EPM_FP_5_2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode=""/>
-  </numFmts>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -98,13 +351,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -142,7 +403,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -176,6 +437,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -210,9 +472,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -385,287 +648,180 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AW12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Trial</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Cagenumber and earmark</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>FP file</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Cohort</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Distance moved Center-point Total cm</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Velocity Center-point Mean cm/s</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>In zone 2 Arena / Center-point Frequency</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>In zone 2 Arena / Center-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>In zone 2 Arena / Center-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>In zone 2 O1_prevC1 / Center-point Frequency</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>In zone 2 O1_prevC1 / Center-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>In zone 2 O1_prevC1 / Center-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>In zone 2 O2_prevC2 / Center-point Frequency</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>In zone 2 O2_prevC2 / Center-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>In zone 2 O2_prevC2 / Center-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>In zone 2 C1_prevO1 / Center-point Frequency</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>In zone 2 C1_prevO1 / Center-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>In zone 2 C1_prevO1 / Center-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>In zone 2 C2_prevO2 / Center-point Frequency</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>In zone 2 C2_prevO2 / Center-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>In zone 2 C2_prevO2 / Center-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>In zone 2 NeutralZone / Center-point Frequency</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>In zone 2 NeutralZone / Center-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>In zone 2 NeutralZone / Center-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>In zone 3 Arena / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>In zone 3 Arena / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>In zone 3 Arena / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>In zone 3 O1_prevC1 / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>In zone 3 O1_prevC1 / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>In zone 3 O1_prevC1 / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>In zone 3 O2_prevC2 / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>In zone 3 O2_prevC2 / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>In zone 3 O2_prevC2 / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>In zone 3 C1_prevO1 / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>In zone 3 C1_prevO1 / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>In zone 3 C1_prevO1 / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>In zone 3 C2_prevO2 / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>In zone 3 C2_prevO2 / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>In zone 3 C2_prevO2 / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>In zone 3 NeutralZone / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>In zone 3 NeutralZone / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>In zone 3 NeutralZone / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>In zone 3 O1_round / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>In zone 3 O1_round / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>In zone 3 O1_round / Nose-point Latency to First s</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>In zone 3 O2_round / Nose-point Frequency</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>In zone 3 O2_round / Nose-point Cumulative Duration s</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>In zone 3 O2_round / Nose-point Latency to First s</t>
-        </is>
+    <row r="1" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Trial     1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>9E10</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>376</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>EPM_FP0_1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="2" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" t="s">
+        <v>53</v>
       </c>
       <c r="F2">
         <v>1189.57</v>
       </c>
       <c r="G2">
-        <v>1.98256</v>
+        <v>1.9825600000000001</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -682,10 +838,8 @@
       <c r="L2">
         <v>0</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="M2" t="s">
+        <v>54</v>
       </c>
       <c r="N2">
         <v>2</v>
@@ -694,7 +848,7 @@
         <v>10.5632</v>
       </c>
       <c r="P2">
-        <v>236.531</v>
+        <v>236.53100000000001</v>
       </c>
       <c r="Q2">
         <v>1</v>
@@ -703,7 +857,7 @@
         <v>351.846</v>
       </c>
       <c r="S2">
-        <v>248.194</v>
+        <v>248.19399999999999</v>
       </c>
       <c r="T2">
         <v>2</v>
@@ -718,16 +872,16 @@
         <v>4</v>
       </c>
       <c r="X2">
-        <v>14.9045</v>
+        <v>14.904500000000001</v>
       </c>
       <c r="Y2">
-        <v>5.54166</v>
+        <v>5.5416600000000003</v>
       </c>
       <c r="Z2">
         <v>163</v>
       </c>
       <c r="AA2">
-        <v>571.411</v>
+        <v>571.41099999999994</v>
       </c>
       <c r="AB2">
         <v>0</v>
@@ -736,10 +890,10 @@
         <v>29</v>
       </c>
       <c r="AD2">
-        <v>35.4706</v>
+        <v>35.470599999999997</v>
       </c>
       <c r="AE2">
-        <v>3.6611</v>
+        <v>3.6610999999999998</v>
       </c>
       <c r="AF2">
         <v>21</v>
@@ -757,13 +911,13 @@
         <v>265.68</v>
       </c>
       <c r="AK2">
-        <v>6.20186</v>
+        <v>6.2018599999999999</v>
       </c>
       <c r="AL2">
         <v>122</v>
       </c>
       <c r="AM2">
-        <v>153.266</v>
+        <v>153.26599999999999</v>
       </c>
       <c r="AN2">
         <v>0</v>
@@ -772,61 +926,51 @@
         <v>87</v>
       </c>
       <c r="AP2">
-        <v>97.5493</v>
+        <v>97.549300000000002</v>
       </c>
       <c r="AQ2">
-        <v>1.26038</v>
+        <v>1.2603800000000001</v>
       </c>
       <c r="AR2">
         <v>1</v>
       </c>
       <c r="AS2">
-        <v>0.020006</v>
+        <v>2.0005999999999999E-2</v>
       </c>
       <c r="AT2">
-        <v>6.48194</v>
+        <v>6.4819399999999998</v>
       </c>
       <c r="AU2">
         <v>3</v>
       </c>
       <c r="AV2">
-        <v>0.060018</v>
+        <v>6.0018000000000002E-2</v>
       </c>
       <c r="AW2">
-        <v>242.013</v>
+        <v>242.01300000000001</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Trial     2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>9E3</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>372</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>EPM_FP1_1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="3" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
+        <v>53</v>
       </c>
       <c r="F3">
         <v>1851.78</v>
       </c>
       <c r="G3">
-        <v>3.0862</v>
+        <v>3.0861999999999998</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -844,7 +988,7 @@
         <v>15.7447</v>
       </c>
       <c r="M3">
-        <v>55.6567</v>
+        <v>55.656700000000001</v>
       </c>
       <c r="N3">
         <v>4</v>
@@ -853,13 +997,13 @@
         <v>10.023</v>
       </c>
       <c r="P3">
-        <v>29.6689</v>
+        <v>29.668900000000001</v>
       </c>
       <c r="Q3">
         <v>12</v>
       </c>
       <c r="R3">
-        <v>242.693</v>
+        <v>242.69300000000001</v>
       </c>
       <c r="S3">
         <v>0</v>
@@ -868,10 +1012,10 @@
         <v>23</v>
       </c>
       <c r="U3">
-        <v>308.372</v>
+        <v>308.37200000000001</v>
       </c>
       <c r="V3">
-        <v>13.344</v>
+        <v>13.343999999999999</v>
       </c>
       <c r="W3">
         <v>53</v>
@@ -886,7 +1030,7 @@
         <v>60</v>
       </c>
       <c r="AA3">
-        <v>585.916</v>
+        <v>585.91600000000005</v>
       </c>
       <c r="AB3">
         <v>0</v>
@@ -907,13 +1051,13 @@
         <v>26.788</v>
       </c>
       <c r="AH3">
-        <v>25.8077</v>
+        <v>25.807700000000001</v>
       </c>
       <c r="AI3">
         <v>42</v>
       </c>
       <c r="AJ3">
-        <v>211.003</v>
+        <v>211.00299999999999</v>
       </c>
       <c r="AK3">
         <v>0</v>
@@ -922,28 +1066,28 @@
         <v>36</v>
       </c>
       <c r="AM3">
-        <v>277.003</v>
+        <v>277.00299999999999</v>
       </c>
       <c r="AN3">
-        <v>12.9639</v>
+        <v>12.963900000000001</v>
       </c>
       <c r="AO3">
         <v>68</v>
       </c>
       <c r="AP3">
-        <v>23.6871</v>
+        <v>23.687100000000001</v>
       </c>
       <c r="AQ3">
-        <v>7.6823</v>
+        <v>7.6822999999999997</v>
       </c>
       <c r="AR3">
         <v>47</v>
       </c>
       <c r="AS3">
-        <v>10.4431</v>
+        <v>10.443099999999999</v>
       </c>
       <c r="AT3">
-        <v>54.7564</v>
+        <v>54.756399999999999</v>
       </c>
       <c r="AU3">
         <v>28</v>
@@ -952,40 +1096,30 @@
         <v>7.18215</v>
       </c>
       <c r="AW3">
-        <v>27.6283</v>
+        <v>27.628299999999999</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Trial     3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>8E4</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>374</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>EPM_FP2_1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="4" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" t="s">
+        <v>53</v>
       </c>
       <c r="F4">
         <v>1896.45</v>
       </c>
       <c r="G4">
-        <v>3.16064</v>
+        <v>3.1606399999999999</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1000,19 +1134,19 @@
         <v>5</v>
       </c>
       <c r="L4">
-        <v>3.78113</v>
+        <v>3.7811300000000001</v>
       </c>
       <c r="M4">
-        <v>261.138</v>
+        <v>261.13799999999998</v>
       </c>
       <c r="N4">
         <v>6</v>
       </c>
       <c r="O4">
-        <v>16.705</v>
+        <v>16.704999999999998</v>
       </c>
       <c r="P4">
-        <v>18.6656</v>
+        <v>18.665600000000001</v>
       </c>
       <c r="Q4">
         <v>6</v>
@@ -1021,7 +1155,7 @@
         <v>133.5</v>
       </c>
       <c r="S4">
-        <v>97.3692</v>
+        <v>97.369200000000006</v>
       </c>
       <c r="T4">
         <v>8</v>
@@ -1030,13 +1164,13 @@
         <v>400.48</v>
       </c>
       <c r="V4">
-        <v>1.30039</v>
+        <v>1.3003899999999999</v>
       </c>
       <c r="W4">
         <v>25</v>
       </c>
       <c r="X4">
-        <v>45.4736</v>
+        <v>45.473599999999998</v>
       </c>
       <c r="Y4">
         <v>0</v>
@@ -1045,7 +1179,7 @@
         <v>115</v>
       </c>
       <c r="AA4">
-        <v>585.836</v>
+        <v>585.83600000000001</v>
       </c>
       <c r="AB4">
         <v>0</v>
@@ -1054,7 +1188,7 @@
         <v>48</v>
       </c>
       <c r="AD4">
-        <v>24.6674</v>
+        <v>24.667400000000001</v>
       </c>
       <c r="AE4">
         <v>15.6647</v>
@@ -1075,13 +1209,13 @@
         <v>116.735</v>
       </c>
       <c r="AK4">
-        <v>93.8281</v>
+        <v>93.828100000000006</v>
       </c>
       <c r="AL4">
         <v>124</v>
       </c>
       <c r="AM4">
-        <v>346.044</v>
+        <v>346.04399999999998</v>
       </c>
       <c r="AN4">
         <v>0</v>
@@ -1090,10 +1224,10 @@
         <v>100</v>
       </c>
       <c r="AP4">
-        <v>44.4333</v>
+        <v>44.433300000000003</v>
       </c>
       <c r="AQ4">
-        <v>11.0833</v>
+        <v>11.083299999999999</v>
       </c>
       <c r="AR4">
         <v>28</v>
@@ -1111,40 +1245,30 @@
         <v>7.64229</v>
       </c>
       <c r="AW4">
-        <v>18.5856</v>
+        <v>18.585599999999999</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Trial     4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>10E13</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>429</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>EPM_FP3_1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" t="s">
+        <v>53</v>
       </c>
       <c r="F5">
-        <v>2502.68</v>
+        <v>2502.6799999999998</v>
       </c>
       <c r="G5">
-        <v>4.171</v>
+        <v>4.1710000000000003</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1159,10 +1283,10 @@
         <v>9</v>
       </c>
       <c r="L5">
-        <v>38.6716</v>
+        <v>38.671599999999998</v>
       </c>
       <c r="M5">
-        <v>63.7591</v>
+        <v>63.759099999999997</v>
       </c>
       <c r="N5">
         <v>8</v>
@@ -1177,7 +1301,7 @@
         <v>12</v>
       </c>
       <c r="R5">
-        <v>312.414</v>
+        <v>312.41399999999999</v>
       </c>
       <c r="S5">
         <v>13.504</v>
@@ -1189,22 +1313,22 @@
         <v>108.092</v>
       </c>
       <c r="V5">
-        <v>28.3885</v>
+        <v>28.388500000000001</v>
       </c>
       <c r="W5">
         <v>41</v>
       </c>
       <c r="X5">
-        <v>57.0571</v>
+        <v>57.057099999999998</v>
       </c>
       <c r="Y5">
-        <v>11.5034</v>
+        <v>11.503399999999999</v>
       </c>
       <c r="Z5">
         <v>144</v>
       </c>
       <c r="AA5">
-        <v>559.208</v>
+        <v>559.20799999999997</v>
       </c>
       <c r="AB5">
         <v>0</v>
@@ -1216,43 +1340,43 @@
         <v>33.31</v>
       </c>
       <c r="AE5">
-        <v>11.9036</v>
+        <v>11.903600000000001</v>
       </c>
       <c r="AF5">
         <v>98</v>
       </c>
       <c r="AG5">
-        <v>64.9995</v>
+        <v>64.999499999999998</v>
       </c>
       <c r="AH5">
-        <v>0.620186</v>
+        <v>0.62018600000000002</v>
       </c>
       <c r="AI5">
         <v>112</v>
       </c>
       <c r="AJ5">
-        <v>280.124</v>
+        <v>280.12400000000002</v>
       </c>
       <c r="AK5">
-        <v>10.6232</v>
+        <v>10.623200000000001</v>
       </c>
       <c r="AL5">
         <v>57</v>
       </c>
       <c r="AM5">
-        <v>86.3859</v>
+        <v>86.385900000000007</v>
       </c>
       <c r="AN5">
-        <v>27.7083</v>
+        <v>27.708300000000001</v>
       </c>
       <c r="AO5">
         <v>88</v>
       </c>
       <c r="AP5">
-        <v>40.7522</v>
+        <v>40.752200000000002</v>
       </c>
       <c r="AQ5">
-        <v>11.3234</v>
+        <v>11.323399999999999</v>
       </c>
       <c r="AR5">
         <v>77</v>
@@ -1261,7 +1385,7 @@
         <v>13.7841</v>
       </c>
       <c r="AT5">
-        <v>63.8191</v>
+        <v>63.819099999999999</v>
       </c>
       <c r="AU5">
         <v>95</v>
@@ -1273,37 +1397,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Trial     5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>10E4</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>423</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>EPM_FP5_1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="6" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s">
+        <v>53</v>
       </c>
       <c r="F6">
         <v>1478.73</v>
       </c>
       <c r="G6">
-        <v>2.46447</v>
+        <v>2.4644699999999999</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -1318,7 +1432,7 @@
         <v>4</v>
       </c>
       <c r="L6">
-        <v>7.98239</v>
+        <v>7.9823899999999997</v>
       </c>
       <c r="M6">
         <v>126.038</v>
@@ -1327,7 +1441,7 @@
         <v>3</v>
       </c>
       <c r="O6">
-        <v>65.4596</v>
+        <v>65.459599999999995</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1338,25 +1452,23 @@
       <c r="R6">
         <v>0</v>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="S6" t="s">
+        <v>54</v>
       </c>
       <c r="T6">
         <v>11</v>
       </c>
       <c r="U6">
-        <v>492.688</v>
+        <v>492.68799999999999</v>
       </c>
       <c r="V6">
-        <v>9.40282</v>
+        <v>9.4028200000000002</v>
       </c>
       <c r="W6">
         <v>17</v>
       </c>
       <c r="X6">
-        <v>33.9102</v>
+        <v>33.910200000000003</v>
       </c>
       <c r="Y6">
         <v>2.64079</v>
@@ -1374,7 +1486,7 @@
         <v>26</v>
       </c>
       <c r="AD6">
-        <v>17.0251</v>
+        <v>17.025099999999998</v>
       </c>
       <c r="AE6">
         <v>2.62079</v>
@@ -1383,7 +1495,7 @@
         <v>62</v>
       </c>
       <c r="AG6">
-        <v>63.479</v>
+        <v>63.478999999999999</v>
       </c>
       <c r="AH6">
         <v>0</v>
@@ -1395,7 +1507,7 @@
         <v>6.36191</v>
       </c>
       <c r="AK6">
-        <v>6.88206</v>
+        <v>6.8820600000000001</v>
       </c>
       <c r="AL6">
         <v>34</v>
@@ -1404,25 +1516,25 @@
         <v>464.339</v>
       </c>
       <c r="AN6">
-        <v>1.74052</v>
+        <v>1.7405200000000001</v>
       </c>
       <c r="AO6">
         <v>45</v>
       </c>
       <c r="AP6">
-        <v>23.487</v>
+        <v>23.486999999999998</v>
       </c>
       <c r="AQ6">
-        <v>1.98059</v>
+        <v>1.9805900000000001</v>
       </c>
       <c r="AR6">
         <v>23</v>
       </c>
       <c r="AS6">
-        <v>5.72172</v>
+        <v>5.7217200000000004</v>
       </c>
       <c r="AT6">
-        <v>5.74172</v>
+        <v>5.7417199999999999</v>
       </c>
       <c r="AU6">
         <v>55</v>
@@ -1434,31 +1546,21 @@
         <v>0.140042</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Trial     6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>8C4</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>461</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>EPM_FP_00_2</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+    <row r="7" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" t="s">
+        <v>75</v>
       </c>
       <c r="F7">
         <v>1678.9</v>
@@ -1470,7 +1572,7 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>600.028</v>
+        <v>600.02800000000002</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -1479,10 +1581,10 @@
         <v>1</v>
       </c>
       <c r="L7">
-        <v>3.96111</v>
+        <v>3.9611100000000001</v>
       </c>
       <c r="M7">
-        <v>378.906</v>
+        <v>378.90600000000001</v>
       </c>
       <c r="N7">
         <v>4</v>
@@ -1497,16 +1599,16 @@
         <v>8</v>
       </c>
       <c r="R7">
-        <v>23.6866</v>
+        <v>23.686599999999999</v>
       </c>
       <c r="S7">
-        <v>301.564</v>
+        <v>301.56400000000002</v>
       </c>
       <c r="T7">
         <v>9</v>
       </c>
       <c r="U7">
-        <v>533.349</v>
+        <v>533.34900000000005</v>
       </c>
       <c r="V7">
         <v>0</v>
@@ -1515,16 +1617,16 @@
         <v>20</v>
       </c>
       <c r="X7">
-        <v>20.6458</v>
+        <v>20.645800000000001</v>
       </c>
       <c r="Y7">
-        <v>5.50154</v>
+        <v>5.5015400000000003</v>
       </c>
       <c r="Z7">
         <v>38</v>
       </c>
       <c r="AA7">
-        <v>597.187</v>
+        <v>597.18700000000001</v>
       </c>
       <c r="AB7">
         <v>0</v>
@@ -1533,34 +1635,34 @@
         <v>12</v>
       </c>
       <c r="AD7">
-        <v>8.12227</v>
+        <v>8.1222700000000003</v>
       </c>
       <c r="AE7">
-        <v>5.30148</v>
+        <v>5.3014799999999997</v>
       </c>
       <c r="AF7">
         <v>39</v>
       </c>
       <c r="AG7">
-        <v>17.0848</v>
+        <v>17.084800000000001</v>
       </c>
       <c r="AH7">
-        <v>6.84191</v>
+        <v>6.8419100000000004</v>
       </c>
       <c r="AI7">
         <v>13</v>
       </c>
       <c r="AJ7">
-        <v>23.9667</v>
+        <v>23.966699999999999</v>
       </c>
       <c r="AK7">
-        <v>4.80134</v>
+        <v>4.8013399999999997</v>
       </c>
       <c r="AL7">
         <v>81</v>
       </c>
       <c r="AM7">
-        <v>495.139</v>
+        <v>495.13900000000001</v>
       </c>
       <c r="AN7">
         <v>0</v>
@@ -1569,61 +1671,51 @@
         <v>55</v>
       </c>
       <c r="AP7">
-        <v>26.2674</v>
+        <v>26.267399999999999</v>
       </c>
       <c r="AQ7">
-        <v>2.06058</v>
+        <v>2.0605799999999999</v>
       </c>
       <c r="AR7">
         <v>7</v>
       </c>
       <c r="AS7">
-        <v>4.3012</v>
+        <v>4.3011999999999997</v>
       </c>
       <c r="AT7">
-        <v>379.466</v>
+        <v>379.46600000000001</v>
       </c>
       <c r="AU7">
         <v>32</v>
       </c>
       <c r="AV7">
-        <v>6.50182</v>
+        <v>6.5018200000000004</v>
       </c>
       <c r="AW7">
-        <v>330.272</v>
+        <v>330.27199999999999</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Trial     7</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>8C10</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>463</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>EPM_FP_0_2</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+    <row r="8" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" t="s">
+        <v>75</v>
       </c>
       <c r="F8">
         <v>1568.26</v>
       </c>
       <c r="G8">
-        <v>2.61369</v>
+        <v>2.6136900000000001</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -1638,10 +1730,10 @@
         <v>2</v>
       </c>
       <c r="L8">
-        <v>3.82115</v>
+        <v>3.8211499999999998</v>
       </c>
       <c r="M8">
-        <v>61.9386</v>
+        <v>61.938600000000001</v>
       </c>
       <c r="N8">
         <v>9</v>
@@ -1656,34 +1748,34 @@
         <v>5</v>
       </c>
       <c r="R8">
-        <v>145.544</v>
+        <v>145.54400000000001</v>
       </c>
       <c r="S8">
-        <v>24.4473</v>
+        <v>24.447299999999998</v>
       </c>
       <c r="T8">
         <v>16</v>
       </c>
       <c r="U8">
-        <v>340.542</v>
+        <v>340.54199999999997</v>
       </c>
       <c r="V8">
-        <v>29.2888</v>
+        <v>29.288799999999998</v>
       </c>
       <c r="W8">
         <v>31</v>
       </c>
       <c r="X8">
-        <v>41.1523</v>
+        <v>41.152299999999997</v>
       </c>
       <c r="Y8">
-        <v>24.2873</v>
+        <v>24.287299999999998</v>
       </c>
       <c r="Z8">
         <v>92</v>
       </c>
       <c r="AA8">
-        <v>589.297</v>
+        <v>589.29700000000003</v>
       </c>
       <c r="AB8">
         <v>0</v>
@@ -1692,19 +1784,19 @@
         <v>18</v>
       </c>
       <c r="AD8">
-        <v>11.1834</v>
+        <v>11.183400000000001</v>
       </c>
       <c r="AE8">
-        <v>25.5477</v>
+        <v>25.547699999999999</v>
       </c>
       <c r="AF8">
         <v>66</v>
       </c>
       <c r="AG8">
-        <v>59.3178</v>
+        <v>59.317799999999998</v>
       </c>
       <c r="AH8">
-        <v>0.340102</v>
+        <v>0.34010200000000002</v>
       </c>
       <c r="AI8">
         <v>71</v>
@@ -1719,7 +1811,7 @@
         <v>87</v>
       </c>
       <c r="AM8">
-        <v>313.594</v>
+        <v>313.59399999999999</v>
       </c>
       <c r="AN8">
         <v>28.5886</v>
@@ -1728,7 +1820,7 @@
         <v>64</v>
       </c>
       <c r="AP8">
-        <v>31.1894</v>
+        <v>31.189399999999999</v>
       </c>
       <c r="AQ8">
         <v>2.50075</v>
@@ -1737,52 +1829,42 @@
         <v>11</v>
       </c>
       <c r="AS8">
-        <v>2.56077</v>
+        <v>2.5607700000000002</v>
       </c>
       <c r="AT8">
-        <v>26.8481</v>
+        <v>26.848099999999999</v>
       </c>
       <c r="AU8">
         <v>61</v>
       </c>
       <c r="AV8">
-        <v>13.204</v>
+        <v>13.204000000000001</v>
       </c>
       <c r="AW8">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Trial     8</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>8C3</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>459</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>EPM_FP_1_2</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+    <row r="9" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" t="s">
+        <v>75</v>
       </c>
       <c r="F9">
         <v>1787.71</v>
       </c>
       <c r="G9">
-        <v>2.97941</v>
+        <v>2.9794100000000001</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1797,7 +1879,7 @@
         <v>2</v>
       </c>
       <c r="L9">
-        <v>9.94298</v>
+        <v>9.9429800000000004</v>
       </c>
       <c r="M9">
         <v>146.084</v>
@@ -1806,34 +1888,34 @@
         <v>6</v>
       </c>
       <c r="O9">
-        <v>19.926</v>
+        <v>19.925999999999998</v>
       </c>
       <c r="P9">
-        <v>215.044</v>
+        <v>215.04400000000001</v>
       </c>
       <c r="Q9">
         <v>18</v>
       </c>
       <c r="R9">
-        <v>460.698</v>
+        <v>460.69799999999998</v>
       </c>
       <c r="S9">
-        <v>0.80024</v>
+        <v>0.80023999999999995</v>
       </c>
       <c r="T9">
         <v>4</v>
       </c>
       <c r="U9">
-        <v>65.2596</v>
+        <v>65.259600000000006</v>
       </c>
       <c r="V9">
-        <v>174.912</v>
+        <v>174.91200000000001</v>
       </c>
       <c r="W9">
         <v>35</v>
       </c>
       <c r="X9">
-        <v>36.571</v>
+        <v>36.570999999999998</v>
       </c>
       <c r="Y9">
         <v>0</v>
@@ -1842,7 +1924,7 @@
         <v>139</v>
       </c>
       <c r="AA9">
-        <v>580.074</v>
+        <v>580.07399999999996</v>
       </c>
       <c r="AB9">
         <v>0</v>
@@ -1851,19 +1933,19 @@
         <v>25</v>
       </c>
       <c r="AD9">
-        <v>11.2434</v>
+        <v>11.243399999999999</v>
       </c>
       <c r="AE9">
-        <v>36.4909</v>
+        <v>36.490900000000003</v>
       </c>
       <c r="AF9">
         <v>60</v>
       </c>
       <c r="AG9">
-        <v>32.0496</v>
+        <v>32.049599999999998</v>
       </c>
       <c r="AH9">
-        <v>3.04091</v>
+        <v>3.0409099999999998</v>
       </c>
       <c r="AI9">
         <v>136</v>
@@ -1872,13 +1954,13 @@
         <v>419.226</v>
       </c>
       <c r="AK9">
-        <v>6.16185</v>
+        <v>6.1618500000000003</v>
       </c>
       <c r="AL9">
         <v>63</v>
       </c>
       <c r="AM9">
-        <v>52.0156</v>
+        <v>52.015599999999999</v>
       </c>
       <c r="AN9">
         <v>0</v>
@@ -1890,52 +1972,42 @@
         <v>20.5061</v>
       </c>
       <c r="AQ9">
-        <v>0.760228</v>
+        <v>0.76022800000000001</v>
       </c>
       <c r="AR9">
         <v>10</v>
       </c>
       <c r="AS9">
-        <v>8.12244</v>
+        <v>8.1224399999999992</v>
       </c>
       <c r="AT9">
-        <v>148.144</v>
+        <v>148.14400000000001</v>
       </c>
       <c r="AU9">
         <v>42</v>
       </c>
       <c r="AV9">
-        <v>16.0648</v>
+        <v>16.064800000000002</v>
       </c>
       <c r="AW9">
-        <v>3.6811</v>
+        <v>3.6810999999999998</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Trial     9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>5B1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>398</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>EPM_FP_3_2</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+    <row r="10" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" t="s">
+        <v>75</v>
       </c>
       <c r="F10">
         <v>1608.04</v>
@@ -1956,7 +2028,7 @@
         <v>2</v>
       </c>
       <c r="L10">
-        <v>12.0836</v>
+        <v>12.083600000000001</v>
       </c>
       <c r="M10">
         <v>1.58047</v>
@@ -1965,25 +2037,25 @@
         <v>16</v>
       </c>
       <c r="O10">
-        <v>24.6274</v>
+        <v>24.627400000000002</v>
       </c>
       <c r="P10">
-        <v>5.10153</v>
+        <v>5.1015300000000003</v>
       </c>
       <c r="Q10">
         <v>14</v>
       </c>
       <c r="R10">
-        <v>247.394</v>
+        <v>247.39400000000001</v>
       </c>
       <c r="S10">
-        <v>16.725</v>
+        <v>16.725000000000001</v>
       </c>
       <c r="T10">
         <v>8</v>
       </c>
       <c r="U10">
-        <v>242.213</v>
+        <v>242.21299999999999</v>
       </c>
       <c r="V10">
         <v>35.8508</v>
@@ -1992,7 +2064,7 @@
         <v>31</v>
       </c>
       <c r="X10">
-        <v>64.8194</v>
+        <v>64.819400000000002</v>
       </c>
       <c r="Y10">
         <v>0</v>
@@ -2001,7 +2073,7 @@
         <v>72</v>
       </c>
       <c r="AA10">
-        <v>589.237</v>
+        <v>589.23699999999997</v>
       </c>
       <c r="AB10">
         <v>0</v>
@@ -2019,28 +2091,28 @@
         <v>44</v>
       </c>
       <c r="AG10">
-        <v>34.5504</v>
+        <v>34.550400000000003</v>
       </c>
       <c r="AH10">
-        <v>4.58137</v>
+        <v>4.5813699999999997</v>
       </c>
       <c r="AI10">
         <v>43</v>
       </c>
       <c r="AJ10">
-        <v>245.674</v>
+        <v>245.67400000000001</v>
       </c>
       <c r="AK10">
-        <v>19.886</v>
+        <v>19.885999999999999</v>
       </c>
       <c r="AL10">
         <v>71</v>
       </c>
       <c r="AM10">
-        <v>230.349</v>
+        <v>230.34899999999999</v>
       </c>
       <c r="AN10">
-        <v>3.50105</v>
+        <v>3.5010500000000002</v>
       </c>
       <c r="AO10">
         <v>43</v>
@@ -2049,52 +2121,42 @@
         <v>13.8241</v>
       </c>
       <c r="AQ10">
-        <v>3.52106</v>
+        <v>3.5210599999999999</v>
       </c>
       <c r="AR10">
         <v>19</v>
       </c>
       <c r="AS10">
-        <v>7.20216</v>
+        <v>7.2021600000000001</v>
       </c>
       <c r="AT10">
-        <v>0.180054</v>
+        <v>0.18005399999999999</v>
       </c>
       <c r="AU10">
         <v>34</v>
       </c>
       <c r="AV10">
-        <v>9.82295</v>
+        <v>9.8229500000000005</v>
       </c>
       <c r="AW10">
-        <v>5.78173</v>
+        <v>5.7817299999999996</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Trial    10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>5B3</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>EPM_FP_4_2</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+    <row r="11" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" t="s">
+        <v>75</v>
       </c>
       <c r="F11">
         <v>1772.16</v>
@@ -2117,10 +2179,8 @@
       <c r="L11">
         <v>0</v>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="M11" t="s">
+        <v>54</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -2128,25 +2188,23 @@
       <c r="O11">
         <v>0</v>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P11" t="s">
+        <v>54</v>
       </c>
       <c r="Q11">
         <v>5</v>
       </c>
       <c r="R11">
-        <v>182.075</v>
+        <v>182.07499999999999</v>
       </c>
       <c r="S11">
-        <v>41.0923</v>
+        <v>41.092300000000002</v>
       </c>
       <c r="T11">
         <v>2</v>
       </c>
       <c r="U11">
-        <v>414.124</v>
+        <v>414.12400000000002</v>
       </c>
       <c r="V11">
         <v>0</v>
@@ -2155,16 +2213,16 @@
         <v>6</v>
       </c>
       <c r="X11">
-        <v>3.76113</v>
+        <v>3.7611300000000001</v>
       </c>
       <c r="Y11">
-        <v>38.2315</v>
+        <v>38.231499999999997</v>
       </c>
       <c r="Z11">
         <v>39</v>
       </c>
       <c r="AA11">
-        <v>596.999</v>
+        <v>596.99900000000002</v>
       </c>
       <c r="AB11">
         <v>0</v>
@@ -2176,31 +2234,31 @@
         <v>2.04061</v>
       </c>
       <c r="AE11">
-        <v>96.3089</v>
+        <v>96.308899999999994</v>
       </c>
       <c r="AF11">
         <v>6</v>
       </c>
       <c r="AG11">
-        <v>2.26068</v>
+        <v>2.2606799999999998</v>
       </c>
       <c r="AH11">
-        <v>36.0708</v>
+        <v>36.070799999999998</v>
       </c>
       <c r="AI11">
         <v>21</v>
       </c>
       <c r="AJ11">
-        <v>171.171</v>
+        <v>171.17099999999999</v>
       </c>
       <c r="AK11">
-        <v>37.6913</v>
+        <v>37.691299999999998</v>
       </c>
       <c r="AL11">
         <v>86</v>
       </c>
       <c r="AM11">
-        <v>395.999</v>
+        <v>395.99900000000002</v>
       </c>
       <c r="AN11">
         <v>0</v>
@@ -2209,10 +2267,10 @@
         <v>46</v>
       </c>
       <c r="AP11">
-        <v>13.184</v>
+        <v>13.183999999999999</v>
       </c>
       <c r="AQ11">
-        <v>29.6089</v>
+        <v>29.608899999999998</v>
       </c>
       <c r="AR11">
         <v>0</v>
@@ -2220,10 +2278,8 @@
       <c r="AS11">
         <v>0</v>
       </c>
-      <c r="AT11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AT11" t="s">
+        <v>54</v>
       </c>
       <c r="AU11">
         <v>0</v>
@@ -2231,37 +2287,25 @@
       <c r="AV11">
         <v>0</v>
       </c>
-      <c r="AW11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AW11" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Trial    11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>5B4</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>402</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>EPM_FP_5_2</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+    <row r="12" spans="1:49" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" t="s">
+        <v>75</v>
       </c>
       <c r="F12">
         <v>1990.45</v>
@@ -2282,7 +2326,7 @@
         <v>1</v>
       </c>
       <c r="L12">
-        <v>0.480144</v>
+        <v>0.48014400000000002</v>
       </c>
       <c r="M12">
         <v>112.914</v>
@@ -2291,7 +2335,7 @@
         <v>6</v>
       </c>
       <c r="O12">
-        <v>27.3682</v>
+        <v>27.368200000000002</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -2300,28 +2344,28 @@
         <v>3</v>
       </c>
       <c r="R12">
-        <v>240.592</v>
+        <v>240.59200000000001</v>
       </c>
       <c r="S12">
-        <v>86.9661</v>
+        <v>86.966099999999997</v>
       </c>
       <c r="T12">
         <v>8</v>
       </c>
       <c r="U12">
-        <v>289.247</v>
+        <v>289.24700000000001</v>
       </c>
       <c r="V12">
-        <v>6.94208</v>
+        <v>6.9420799999999998</v>
       </c>
       <c r="W12">
         <v>25</v>
       </c>
       <c r="X12">
-        <v>35.2906</v>
+        <v>35.290599999999998</v>
       </c>
       <c r="Y12">
-        <v>4.04121</v>
+        <v>4.0412100000000004</v>
       </c>
       <c r="Z12">
         <v>111</v>
@@ -2336,7 +2380,7 @@
         <v>8</v>
       </c>
       <c r="AD12">
-        <v>3.24097</v>
+        <v>3.2409699999999999</v>
       </c>
       <c r="AE12">
         <v>109.633</v>
@@ -2345,43 +2389,43 @@
         <v>40</v>
       </c>
       <c r="AG12">
-        <v>26.2679</v>
+        <v>26.267900000000001</v>
       </c>
       <c r="AH12">
-        <v>0.440132</v>
+        <v>0.44013200000000002</v>
       </c>
       <c r="AI12">
         <v>88</v>
       </c>
       <c r="AJ12">
-        <v>228.188</v>
+        <v>228.18799999999999</v>
       </c>
       <c r="AK12">
-        <v>85.9058</v>
+        <v>85.905799999999999</v>
       </c>
       <c r="AL12">
         <v>84</v>
       </c>
       <c r="AM12">
-        <v>282.965</v>
+        <v>282.96499999999997</v>
       </c>
       <c r="AN12">
-        <v>3.38101</v>
+        <v>3.3810099999999998</v>
       </c>
       <c r="AO12">
         <v>44</v>
       </c>
       <c r="AP12">
-        <v>7.38221</v>
+        <v>7.3822099999999997</v>
       </c>
       <c r="AQ12">
-        <v>3.341</v>
+        <v>3.3410000000000002</v>
       </c>
       <c r="AR12">
         <v>15</v>
       </c>
       <c r="AS12">
-        <v>8.6626</v>
+        <v>8.6625999999999994</v>
       </c>
       <c r="AT12">
         <v>110.253</v>
@@ -2401,25 +2445,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <KMRead xmlns="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a">false</KMRead>
+    <TaxCatchAll xmlns="7e264fe7-6d25-4ff1-8e4e-4c598014396b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010093A71806A9E2F349A82303FCAE9EB714" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10df241ec830d831b0ecc6b81b7eb37e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a" xmlns:ns3="7e264fe7-6d25-4ff1-8e4e-4c598014396b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4d2ae054dd02b5abbd3856dbac506afd" ns2:_="" ns3:_="">
     <xsd:import namespace="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a"/>
@@ -2666,35 +2713,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <KMRead xmlns="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a">false</KMRead>
-    <TaxCatchAll xmlns="7e264fe7-6d25-4ff1-8e4e-4c598014396b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D59B7C9C-EDC0-4AC9-B864-61620C8CB700}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B07C3350-583B-46DF-9067-81EA32952A1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a"/>
+    <ds:schemaRef ds:uri="7e264fe7-6d25-4ff1-8e4e-4c598014396b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B4949B8-F193-42D1-847E-C777480CC7F2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B4949B8-F193-42D1-847E-C777480CC7F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B07C3350-583B-46DF-9067-81EA32952A1D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D59B7C9C-EDC0-4AC9-B864-61620C8CB700}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a6d3ddc5-3d2f-43cf-8084-4bb1cb39b18a"/>
+    <ds:schemaRef ds:uri="7e264fe7-6d25-4ff1-8e4e-4c598014396b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>